<commit_message>
fix(excel): remove link column from highlight workbooks
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/exports/day-2026-10-17-en.xlsx
+++ b/docs/exports/day-2026-10-17-en.xlsx
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -38,12 +38,6 @@
       <b val="1"/>
       <color rgb="001F6B56"/>
       <sz val="12"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <color rgb="001F6B56"/>
-      <sz val="11"/>
-      <u val="single"/>
     </font>
   </fonts>
   <fills count="4">
@@ -86,7 +80,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -98,17 +92,11 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -476,12 +464,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:C12"/>
+  <dimension ref="A1:B12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="88" customWidth="1" min="2" max="2"/>
-    <col width="11" customWidth="1" min="3" max="3"/>
+    <col width="92" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1" ht="40" customHeight="1">
@@ -494,9 +481,8 @@
     <row r="2" ht="6" customHeight="1">
       <c r="A2" s="2" t="n"/>
       <c r="B2" s="2" t="n"/>
-      <c r="C2" s="2" t="n"/>
-    </row>
-    <row r="3" ht="98" customHeight="1">
+    </row>
+    <row r="3" ht="78" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
           <t>01</t>
@@ -532,13 +518,8 @@
           </r>
         </is>
       </c>
-      <c r="C3" s="5" t="inlineStr">
-        <is>
-          <t>Open ›</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="114" customHeight="1">
+    </row>
+    <row r="4" ht="78" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
           <t>02</t>
@@ -574,13 +555,8 @@
           </r>
         </is>
       </c>
-      <c r="C4" s="5" t="inlineStr">
-        <is>
-          <t>Open ›</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="94" customHeight="1">
+    </row>
+    <row r="5" ht="78" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
           <t>03</t>
@@ -616,19 +592,14 @@
           </r>
         </is>
       </c>
-      <c r="C5" s="5" t="inlineStr">
-        <is>
-          <t>Open ›</t>
-        </is>
-      </c>
     </row>
     <row r="6" ht="98" customHeight="1">
-      <c r="A6" s="6" t="inlineStr">
+      <c r="A6" s="5" t="inlineStr">
         <is>
           <t>04</t>
         </is>
       </c>
-      <c r="B6" s="7" t="inlineStr">
+      <c r="B6" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -658,19 +629,14 @@
           </r>
         </is>
       </c>
-      <c r="C6" s="8" t="inlineStr">
-        <is>
-          <t>Open ›</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="114" customHeight="1">
-      <c r="A7" s="6" t="inlineStr">
+    </row>
+    <row r="7" ht="94" customHeight="1">
+      <c r="A7" s="5" t="inlineStr">
         <is>
           <t>05</t>
         </is>
       </c>
-      <c r="B7" s="7" t="inlineStr">
+      <c r="B7" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -700,19 +666,14 @@
           </r>
         </is>
       </c>
-      <c r="C7" s="8" t="inlineStr">
-        <is>
-          <t>Open ›</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="114" customHeight="1">
-      <c r="A8" s="6" t="inlineStr">
+    </row>
+    <row r="8" ht="78" customHeight="1">
+      <c r="A8" s="5" t="inlineStr">
         <is>
           <t>06</t>
         </is>
       </c>
-      <c r="B8" s="7" t="inlineStr">
+      <c r="B8" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -742,19 +703,14 @@
           </r>
         </is>
       </c>
-      <c r="C8" s="8" t="inlineStr">
-        <is>
-          <t>Open ›</t>
-        </is>
-      </c>
     </row>
     <row r="9" ht="98" customHeight="1">
-      <c r="A9" s="6" t="inlineStr">
+      <c r="A9" s="5" t="inlineStr">
         <is>
           <t>07</t>
         </is>
       </c>
-      <c r="B9" s="7" t="inlineStr">
+      <c r="B9" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -784,19 +740,14 @@
           </r>
         </is>
       </c>
-      <c r="C9" s="8" t="inlineStr">
-        <is>
-          <t>Open ›</t>
-        </is>
-      </c>
     </row>
     <row r="10" ht="98" customHeight="1">
-      <c r="A10" s="6" t="inlineStr">
+      <c r="A10" s="5" t="inlineStr">
         <is>
           <t>08</t>
         </is>
       </c>
-      <c r="B10" s="7" t="inlineStr">
+      <c r="B10" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -826,19 +777,14 @@
           </r>
         </is>
       </c>
-      <c r="C10" s="8" t="inlineStr">
-        <is>
-          <t>Open ›</t>
-        </is>
-      </c>
     </row>
     <row r="11" ht="98" customHeight="1">
-      <c r="A11" s="6" t="inlineStr">
+      <c r="A11" s="5" t="inlineStr">
         <is>
           <t>09</t>
         </is>
       </c>
-      <c r="B11" s="7" t="inlineStr">
+      <c r="B11" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -868,19 +814,14 @@
           </r>
         </is>
       </c>
-      <c r="C11" s="8" t="inlineStr">
-        <is>
-          <t>Open ›</t>
-        </is>
-      </c>
     </row>
     <row r="12" ht="98" customHeight="1">
-      <c r="A12" s="6" t="inlineStr">
+      <c r="A12" s="5" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="B12" s="7" t="inlineStr">
+      <c r="B12" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -908,30 +849,13 @@
             </rPr>
             <t>Vietnam’s government news portal reported October 3 that estimated realized FDI reached $21.07 billion in the first nine months, up 12.1% yearly, while total registered foreign investment reached $50.36 billion, up 76.4%. This is regional background through September 30, not a new October 17 release.</t>
           </r>
-        </is>
-      </c>
-      <c r="C12" s="8" t="inlineStr">
-        <is>
-          <t>Open ›</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A1:B1"/>
   </mergeCells>
-  <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C3" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C4" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C5" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C6" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C7" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C8" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C9" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C10" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C11" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C12" r:id="rId10"/>
-  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" fitToHeight="0" fitToWidth="1"/>
 </worksheet>

</xml_diff>

<commit_message>
feat(excel): combine summary and full sheets in daily and weekly workbooks
The summary alone could hide the key facts. Each workbook now adds a
full sheet with the complete reading paragraph, including industry
context, location, figures and caveats, beside the summary sheet.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/exports/day-2026-10-17-en.xlsx
+++ b/docs/exports/day-2026-10-17-en.xlsx
@@ -7,10 +7,12 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Highlights" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Full" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Titles" localSheetId="0">'Highlights'!$1:$2</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="0">'Summary'!$1:$2</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="1">'Full'!$1:$2</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -859,4 +861,408 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="007A8780"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:B12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="92" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="40" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Daily Brief highlights · 2026-10-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="6" customHeight="1">
+      <c r="A2" s="2" t="n"/>
+      <c r="B2" s="2" t="n"/>
+    </row>
+    <row r="3" ht="254" customHeight="1">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="0014322B"/>
+              <sz val="13"/>
+            </rPr>
+            <t>Weekly follow-up: TSMC CoWoS production and Micron’s Taichung HBM assembly/test opening</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="007A8780"/>
+              <sz val="11"/>
+            </rPr>
+            <t xml:space="preserve">   Oct 17
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="003B4A44"/>
+              <sz val="11"/>
+            </rPr>
+            <t>TSMC said on October 15 that its five-reticle CoWoS platform was in production. Micron opened its Taichung AATT2 advanced assembly and test facility for HBM the same day. These are weekly follow-ups; no new capacity figures are established today. Location: Micron opening: AATT2 advanced assembly and test facility, Taichung, Taiwan. AI designs move through wafer fabrication, packaging with HBM, testing and server assembly. Yield or delivery constraints at any layer can limit systems output; announced expansions cannot simply be added together. HBM serves accelerator packages, server DRAM system memory, and NAND and enterprise SSDs storage. TrendForce’s September 30 research describes stronger server and enterprise SSD demand alongside cautious consumer purchasing. This background forecast does not establish universal profit growth. Upstream checks include etch, deposition and equipment power; downstream checks include substrates, bonding, probes, burn-in and reliability. TrendForce’s October 13 mapping identifies Taiwanese testing or assembly roles including MPI, WinWay, Chroma and ASE. It does not establish new orders for these events. Added AATT2 HBM output, tool orders and individual supplier revenue are undisclosed. TSMC reported Q3 revenue of US$46.72 billion and a 66.4% gross margin. Taiwan-dollar revenue was about NT$1.494 trillion, up 50.9% annually, and net income NT$763.06 billion, up 68.7%. Growth rates in different currencies must remain distinct. These results were released October 15. From wafers to backend delivery: CoWoS / HBM. Verification confidence: High.</t>
+          </r>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="254" customHeight="1">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>02</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="0014322B"/>
+              <sz val="13"/>
+            </rPr>
+            <t>Taiwan vendors exhibit racks, 800 VDC power and liquid cooling at OCP in San Jose</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="007A8780"/>
+              <sz val="11"/>
+            </rPr>
+            <t xml:space="preserve">   Oct 17
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="003B4A44"/>
+              <sz val="11"/>
+            </rPr>
+            <t>CNA’s October 17 roundup of the October 12–15 OCP summit in San Jose, California describes server or rack exhibits from Wiwynn, ASUS and Chenbro, alongside power systems from Delta, Lite-On and AcBel. Delta’s October 15 release details 800 VDC power, backup and liquid cooling products. Exhibits are distinct from production deployments. Location: San Jose McEnery Convention Center, San Jose, California, United States. OCP Global Summit 2026 ran October 12–15 local time in San Jose, California, at the San Jose McEnery Convention Center. Coverage follows Taiwanese exhibitors; the event location does not imply that their production or investment is located in the United States. Chips, HBM and packaging still need boards, networking, mechanics, power, backup, cooling and system testing. Availability and site power affect customer acceptance; compute specifications cover only part of delivery. Delta, Lite-On and AcBel exhibits make high-voltage DC design and integration comparable topics. Comparable costs, efficiency curves and production orders are unavailable, preventing market-share conclusions; product specifications and customer qualifications need separate comparisons. Delta lists a 660 kW power rack and 480 kW backup rating. These are product capabilities, not deployed customer consumption or sold capacity. The 800 V architecture is not an energy-saving percentage. Comparable prices, costs, customer orders and deployed volumes are undisclosed. Exhibited power architecture: 800 VDC. Verification confidence: High.</t>
+          </r>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="190" customHeight="1">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>03</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="0014322B"/>
+              <sz val="13"/>
+            </rPr>
+            <t>Ho Chi Minh City seeks clarity on AI data-center power tariffs</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="007A8780"/>
+              <sz val="11"/>
+            </rPr>
+            <t xml:space="preserve">   Oct 17
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="003B4A44"/>
+              <sz val="11"/>
+            </rPr>
+            <t>TNGlobal reported October 16 that Ho Chi Minh City’s industrial-zone authority sought unified AI data-center power-tariff guidance at an October 15 meeting. The AIC–KBC project, with a planned $2.1 billion investment, was announced in March. The new development is tariff clarification, not a new investment announcement. Location: Ho Chi Minh City, Vietnam; project at Tan Phu Trung Industrial Park. The issue is business versus manufacturing tariffs. Higher tariffs could affect costs, feasibility and timing. Final rates, load profiles and a financial model are unavailable, preventing a quantified cost difference. Original meeting records, final tariffs, load profiles and power contracts are unavailable. TNGlobal describes phase-one plans of up to 50 MW, while $2.1 billion refers to the previously announced overall project. Their scope and timing are not fully aligned. No per-MW construction cost is calculated from these figures, and planned capacity is not energized or leased capacity. Previously announced project amount: US$2.1B. Verification confidence: Medium.</t>
+          </r>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="178" customHeight="1">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>04</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="0014322B"/>
+              <sz val="13"/>
+            </rPr>
+            <t>Background follow-up: NVIDIA announces semiconductor inspection, testing and factory AI collaborations</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="007A8780"/>
+              <sz val="11"/>
+            </rPr>
+            <t xml:space="preserve">   Oct 17
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="003B4A44"/>
+              <sz val="11"/>
+            </rPr>
+            <t>NVIDIA’s October 14 release describes KLA inspection, Advantest testing and factory AI collaborations involving Foxconn and FANUC. This is background for Taiwan-linked supply chains and end-use factories; deployment sites, full production schedules and plant-wide ROI are not fully disclosed. Location: Global collaboration announcement; individual factory deployment sites are not fully disclosed. Chips and servers provide compute, inspection and test tools generate data, and factories connect models to engineering, scheduling or operations. Partnership lists indicate possible interfaces; they do not establish complete integration or transferability across plants. Named deployment sites, contract pricing and quantified plant-wide benefits are incompletely disclosed. Track adoption; no verified plant-wide returns: 試點與驗收. Verification confidence: Medium.</t>
+          </r>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="222" customHeight="1">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>05</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="0014322B"/>
+              <sz val="13"/>
+            </rPr>
+            <t>Malaysia semiconductor recruitment spans process, equipment and facilities roles</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="007A8780"/>
+              <sz val="11"/>
+            </rPr>
+            <t xml:space="preserve">   Oct 17
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="003B4A44"/>
+              <sz val="11"/>
+            </rPr>
+            <t>CNA reported October 16 that a semiconductor recruitment event organized by Selangor-linked institutions at KLCC in Kuala Lumpur offered over 1,500 vacancies across design, software, firmware, process, equipment and facilities. An official reported 20 companies and 409 engineers in two design parks, complementing Penang manufacturing, assembly and testing. Location: Kuala Lumpur Convention Centre (KLCC), Kuala Lumpur, Malaysia; organized by Selangor-linked institutions. The recruitment venue is KLCC in Kuala Lumpur, Malaysia, distinct from the organizing state of Selangor. Sidec and CNA list October 14–17, while ASEM’s recruitment page lists October 15–17. The venue agrees, but the subevent start date differs; that discrepancy is retained. Backend operations require process, test, maintenance and facilities staff; design clusters also need customers and manufacturing partners. Vacancies signal recruiting demand, not realized hires, output or payroll. Actual hiring and retention are undisclosed; park and program figures are official statements. CNA quoted an official describing a RM150 million program involving Selangor, Penang and the national investment institution. Current disbursement, foreign-capital share and funding timing are not listed; program size differs from new FDI flows. Advertised vacancies, not hires: &gt;1,500. Verification confidence: Medium.</t>
+          </r>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="174" customHeight="1">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>06</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="0014322B"/>
+              <sz val="13"/>
+            </rPr>
+            <t>AUO targets glass and optical components; pure-panel revenue share goal is 30% by 2030</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="007A8780"/>
+              <sz val="11"/>
+            </rPr>
+            <t xml:space="preserve">   Oct 17
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="003B4A44"/>
+              <sz val="11"/>
+            </rPr>
+            <t>AUO chairman Paul Peng said on October 17 that the company would supply advanced-packaging components using glass and TGV expertise. Technology developed with Corning already has low-earth-orbit antenna applications. A two-to-three-year volume-production outlook for MicroLED optical communications and CPO remains a company forecast. Glass processing can extend into new components, but packaging reliability, flatness and production yield require qualification. Progress in satellite applications does not establish semiconductor-packaging acceptance. The 30% figure is a targeted revenue mix in 2030, not a 30% revenue decline. Coverage relies on CNA’s named interview; transcripts, customer qualification and profitability evidence were unavailable. Source-limited. Pure-panel revenue share target: 2030 / 30%. Verification confidence: Medium. New-business profitability, customer qualifications and a full transcript are unavailable.</t>
+          </r>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="146" customHeight="1">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>07</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="0014322B"/>
+              <sz val="13"/>
+            </rPr>
+            <t>RTX Spark PCs launch October 16, connecting Taiwan design, packaging and brands to local AI</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="007A8780"/>
+              <sz val="11"/>
+            </rPr>
+            <t xml:space="preserve">   Oct 17
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="003B4A44"/>
+              <sz val="11"/>
+            </rPr>
+            <t>NVIDIA announced RTX Spark Windows PCs on October 16, with ASUS, MSI and international PC brands using Grace CPUs and Blackwell GPUs. An executive told CNA that MediaTek contributed CPU design and that the platform uses CoWoS; demand and capacity assessments remain company statements. NVIDIA lists Grace CPUs, Blackwell GPUs and brands including ASUS and MSI. An executive told CNA that MediaTek contributed CPU design and the platform uses CoWoS; this edition does not establish HBM content. Shipments, utilization and full lifecycle costs are unavailable in this edition. Company-stated maximum unified memory: 128 GB. Verification confidence: High.</t>
+          </r>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="178" customHeight="1">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>08</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="0014322B"/>
+              <sz val="13"/>
+            </rPr>
+            <t>Taiwan says planned U.S. parks would be privately funded at an estimated $2–4 billion each</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="007A8780"/>
+              <sz val="11"/>
+            </rPr>
+            <t xml:space="preserve">   Oct 17
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="003B4A44"/>
+              <sz val="11"/>
+            </rPr>
+            <t>Taiwan’s economics ministry told CNA on October 16 that it would work with TEEMA on privately funded overseas industrial parks. Minister Kung Ming-hsin described starting in Texas; the estimated $2–4 billion per park is a plan, with land details unconfirmed. Location: Investment plan: Texas, United States; specific park land remains unconfirmed. The ministry described private funding with government assistance and TEEMA participation. Plans would start in Texas and involve more than one park, at an estimated $2–4 billion per park. The estimate comes from the minister and ministry statements reported by media. Full financing, budget and land documents were unavailable; it is neither appropriated government spending nor fully committed capital. Developer, land, complete financing and tenant lists are unconfirmed. Planning estimate per park: US$2–4B. Verification confidence: Medium.</t>
+          </r>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="178" customHeight="1">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>09</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="0014322B"/>
+              <sz val="13"/>
+            </rPr>
+            <t>CIER raises Taiwan’s full-year growth forecast to 12.16%; distinguish results from projections</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="007A8780"/>
+              <sz val="11"/>
+            </rPr>
+            <t xml:space="preserve">   Oct 17
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="003B4A44"/>
+              <sz val="11"/>
+            </rPr>
+            <t>CIER’s October 16 forecast raised 2026 growth from July’s 10.35% to 12.16%, an increase of 1.81 percentage points. Domestic demand is projected to contribute 6.63 points and net external demand 5.53; the full-year figure remains a forecast. The two figures are different vintages of the same-year forecast, separated by 1.81 percentage points. Fourth-quarter growth is projected at 8.20% against a high prior-year base; slower growth does not itself mean output contracts. CIER cited AI demand, corporate expansion and domestic investment as forecast drivers, alongside financing, geopolitical and AI-cybersecurity uncertainties. These are the institution’s assumptions for its full-year forecast. Full-year GDP remains a forecast, subject to subsequent actual data. CIER 2026 full-year GDP growth forecast: 12.16%. Verification confidence: High.</t>
+          </r>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="226" customHeight="1">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="0014322B"/>
+              <sz val="13"/>
+            </rPr>
+            <t>Regional background: Vietnam nine-month realized FDI rises 12.1%; distinguish registrations from execution</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="007A8780"/>
+              <sz val="11"/>
+            </rPr>
+            <t xml:space="preserve">   Oct 17
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="003B4A44"/>
+              <sz val="11"/>
+            </rPr>
+            <t>Vietnam’s government news portal reported October 3 that estimated realized FDI reached $21.07 billion in the first nine months, up 12.1% yearly, while total registered foreign investment reached $50.36 billion, up 76.4%. This is regional background through September 30, not a new October 17 release. Location: Nationwide Vietnam statistics; not a single event or factory. Registrations include new projects, additions and equity transactions, while realized FDI uses a different scope. They cannot be added, and the ratio is not a project completion rate because cohorts differ. Comparable prior-year amounts are not provided. Manufacturing and investor-origin details lack original-table verification; realized FDI is estimated. VnEconomy reported October 4 that manufacturing and processing received $21.82 billion, or 50.3% of new and additional registrations. Singapore supplied $9.26 billion, or 31.7% of newly registered capital. Neither percentage uses the $50.36 billion total-registration denominator. These breakdowns have not been checked against original official tables and are source-limited. Nine-month realized FDI growth: 12.1% YoY. Verification confidence: Medium: official totals; added breakdowns await original-table verification.</t>
+          </r>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:B1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" fitToHeight="0" fitToWidth="1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
feat: show event dates separately from the edition date
Every story showed the edition date 10/17, although several reported
events from earlier days (for example 10/3 and 10/15). Headlines now
show the event date, and workbooks give it its own typed date column.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/exports/day-2026-10-17-en.xlsx
+++ b/docs/exports/day-2026-10-17-en.xlsx
@@ -20,8 +20,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="3">
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="165" formatCode="mmm d"/>
+  </numFmts>
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -38,8 +41,20 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
+      <color rgb="007A8780"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
       <color rgb="001F6B56"/>
       <sz val="12"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="003B4A44"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="4">
@@ -82,23 +97,34 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="4" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -466,11 +492,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:B12"/>
+  <dimension ref="A1:C12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="92" customWidth="1" min="2" max="2"/>
+    <col width="86" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1" ht="40" customHeight="1">
@@ -480,34 +507,39 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="6" customHeight="1">
-      <c r="A2" s="2" t="n"/>
-      <c r="B2" s="2" t="n"/>
-    </row>
-    <row r="3" ht="78" customHeight="1">
-      <c r="A3" s="3" t="inlineStr">
+    <row r="2" ht="22" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>Story</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Event date</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="82" customHeight="1">
+      <c r="A3" s="4" t="inlineStr">
         <is>
           <t>01</t>
         </is>
       </c>
-      <c r="B3" s="4" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <b val="1"/>
-              <color rgb="0014322B"/>
-              <sz val="13"/>
-            </rPr>
-            <t>Weekly follow-up: TSMC CoWoS production and Micron’s Taichung HBM assembly/test opening</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <color rgb="007A8780"/>
-              <sz val="11"/>
-            </rPr>
-            <t xml:space="preserve">   Oct 17
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="0014322B"/>
+              <sz val="13"/>
+            </rPr>
+            <t xml:space="preserve">Weekly follow-up: TSMC CoWoS production and Micron’s Taichung HBM assembly/test opening
 </t>
           </r>
           <r>
@@ -520,31 +552,26 @@
           </r>
         </is>
       </c>
-    </row>
-    <row r="4" ht="78" customHeight="1">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="C3" s="6" t="n">
+        <v>46310</v>
+      </c>
+    </row>
+    <row r="4" ht="98" customHeight="1">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>02</t>
         </is>
       </c>
-      <c r="B4" s="4" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <b val="1"/>
-              <color rgb="0014322B"/>
-              <sz val="13"/>
-            </rPr>
-            <t>Taiwan vendors exhibit racks, 800 VDC power and liquid cooling at OCP in San Jose</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <color rgb="007A8780"/>
-              <sz val="11"/>
-            </rPr>
-            <t xml:space="preserve">   Oct 17
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="0014322B"/>
+              <sz val="13"/>
+            </rPr>
+            <t xml:space="preserve">Taiwan vendors exhibit racks, 800 VDC power and liquid cooling at OCP in San Jose
 </t>
           </r>
           <r>
@@ -557,31 +584,26 @@
           </r>
         </is>
       </c>
-    </row>
-    <row r="5" ht="78" customHeight="1">
-      <c r="A5" s="3" t="inlineStr">
+      <c r="C4" s="6" t="n">
+        <v>46310</v>
+      </c>
+    </row>
+    <row r="5" ht="82" customHeight="1">
+      <c r="A5" s="4" t="inlineStr">
         <is>
           <t>03</t>
         </is>
       </c>
-      <c r="B5" s="4" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <b val="1"/>
-              <color rgb="0014322B"/>
-              <sz val="13"/>
-            </rPr>
-            <t>Ho Chi Minh City seeks clarity on AI data-center power tariffs</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <color rgb="007A8780"/>
-              <sz val="11"/>
-            </rPr>
-            <t xml:space="preserve">   Oct 17
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="0014322B"/>
+              <sz val="13"/>
+            </rPr>
+            <t xml:space="preserve">Ho Chi Minh City seeks clarity on AI data-center power tariffs
 </t>
           </r>
           <r>
@@ -594,31 +616,26 @@
           </r>
         </is>
       </c>
-    </row>
-    <row r="6" ht="98" customHeight="1">
-      <c r="A6" s="5" t="inlineStr">
+      <c r="C5" s="6" t="n">
+        <v>46310</v>
+      </c>
+    </row>
+    <row r="6" ht="102" customHeight="1">
+      <c r="A6" s="7" t="inlineStr">
         <is>
           <t>04</t>
         </is>
       </c>
-      <c r="B6" s="6" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <b val="1"/>
-              <color rgb="0014322B"/>
-              <sz val="13"/>
-            </rPr>
-            <t>Background follow-up: NVIDIA announces semiconductor inspection, testing and factory AI collaborations</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <color rgb="007A8780"/>
-              <sz val="11"/>
-            </rPr>
-            <t xml:space="preserve">   Oct 17
+      <c r="B6" s="8" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="0014322B"/>
+              <sz val="13"/>
+            </rPr>
+            <t xml:space="preserve">Background follow-up: NVIDIA announces semiconductor inspection, testing and factory AI collaborations
 </t>
           </r>
           <r>
@@ -631,31 +648,26 @@
           </r>
         </is>
       </c>
-    </row>
-    <row r="7" ht="94" customHeight="1">
-      <c r="A7" s="5" t="inlineStr">
+      <c r="C6" s="9" t="n">
+        <v>46309</v>
+      </c>
+    </row>
+    <row r="7" ht="98" customHeight="1">
+      <c r="A7" s="7" t="inlineStr">
         <is>
           <t>05</t>
         </is>
       </c>
-      <c r="B7" s="6" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <b val="1"/>
-              <color rgb="0014322B"/>
-              <sz val="13"/>
-            </rPr>
-            <t>Malaysia semiconductor recruitment spans process, equipment and facilities roles</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <color rgb="007A8780"/>
-              <sz val="11"/>
-            </rPr>
-            <t xml:space="preserve">   Oct 17
+      <c r="B7" s="8" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="0014322B"/>
+              <sz val="13"/>
+            </rPr>
+            <t xml:space="preserve">Malaysia semiconductor recruitment spans process, equipment and facilities roles
 </t>
           </r>
           <r>
@@ -668,31 +680,26 @@
           </r>
         </is>
       </c>
-    </row>
-    <row r="8" ht="78" customHeight="1">
-      <c r="A8" s="5" t="inlineStr">
+      <c r="C7" s="9" t="n">
+        <v>46311</v>
+      </c>
+    </row>
+    <row r="8" ht="98" customHeight="1">
+      <c r="A8" s="7" t="inlineStr">
         <is>
           <t>06</t>
         </is>
       </c>
-      <c r="B8" s="6" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <b val="1"/>
-              <color rgb="0014322B"/>
-              <sz val="13"/>
-            </rPr>
-            <t>AUO targets glass and optical components; pure-panel revenue share goal is 30% by 2030</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <color rgb="007A8780"/>
-              <sz val="11"/>
-            </rPr>
-            <t xml:space="preserve">   Oct 17
+      <c r="B8" s="8" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="0014322B"/>
+              <sz val="13"/>
+            </rPr>
+            <t xml:space="preserve">AUO targets glass and optical components; pure-panel revenue share goal is 30% by 2030
 </t>
           </r>
           <r>
@@ -705,31 +712,26 @@
           </r>
         </is>
       </c>
-    </row>
-    <row r="9" ht="98" customHeight="1">
-      <c r="A9" s="5" t="inlineStr">
+      <c r="C8" s="9" t="n">
+        <v>46312</v>
+      </c>
+    </row>
+    <row r="9" ht="102" customHeight="1">
+      <c r="A9" s="7" t="inlineStr">
         <is>
           <t>07</t>
         </is>
       </c>
-      <c r="B9" s="6" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <b val="1"/>
-              <color rgb="0014322B"/>
-              <sz val="13"/>
-            </rPr>
-            <t>RTX Spark PCs launch October 16, connecting Taiwan design, packaging and brands to local AI</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <color rgb="007A8780"/>
-              <sz val="11"/>
-            </rPr>
-            <t xml:space="preserve">   Oct 17
+      <c r="B9" s="8" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="0014322B"/>
+              <sz val="13"/>
+            </rPr>
+            <t xml:space="preserve">RTX Spark PCs launch October 16, connecting Taiwan design, packaging and brands to local AI
 </t>
           </r>
           <r>
@@ -742,31 +744,26 @@
           </r>
         </is>
       </c>
-    </row>
-    <row r="10" ht="98" customHeight="1">
-      <c r="A10" s="5" t="inlineStr">
+      <c r="C9" s="9" t="n">
+        <v>46311</v>
+      </c>
+    </row>
+    <row r="10" ht="82" customHeight="1">
+      <c r="A10" s="7" t="inlineStr">
         <is>
           <t>08</t>
         </is>
       </c>
-      <c r="B10" s="6" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <b val="1"/>
-              <color rgb="0014322B"/>
-              <sz val="13"/>
-            </rPr>
-            <t>Taiwan says planned U.S. parks would be privately funded at an estimated $2–4 billion each</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <color rgb="007A8780"/>
-              <sz val="11"/>
-            </rPr>
-            <t xml:space="preserve">   Oct 17
+      <c r="B10" s="8" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="0014322B"/>
+              <sz val="13"/>
+            </rPr>
+            <t xml:space="preserve">Taiwan says planned U.S. parks would be privately funded at an estimated $2–4 billion each
 </t>
           </r>
           <r>
@@ -779,31 +776,26 @@
           </r>
         </is>
       </c>
-    </row>
-    <row r="11" ht="98" customHeight="1">
-      <c r="A11" s="5" t="inlineStr">
+      <c r="C10" s="9" t="n">
+        <v>46311</v>
+      </c>
+    </row>
+    <row r="11" ht="102" customHeight="1">
+      <c r="A11" s="7" t="inlineStr">
         <is>
           <t>09</t>
         </is>
       </c>
-      <c r="B11" s="6" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <b val="1"/>
-              <color rgb="0014322B"/>
-              <sz val="13"/>
-            </rPr>
-            <t>CIER raises Taiwan’s full-year growth forecast to 12.16%; distinguish results from projections</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <color rgb="007A8780"/>
-              <sz val="11"/>
-            </rPr>
-            <t xml:space="preserve">   Oct 17
+      <c r="B11" s="8" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="0014322B"/>
+              <sz val="13"/>
+            </rPr>
+            <t xml:space="preserve">CIER raises Taiwan’s full-year growth forecast to 12.16%; distinguish results from projections
 </t>
           </r>
           <r>
@@ -816,31 +808,26 @@
           </r>
         </is>
       </c>
-    </row>
-    <row r="12" ht="98" customHeight="1">
-      <c r="A12" s="5" t="inlineStr">
+      <c r="C11" s="9" t="n">
+        <v>46311</v>
+      </c>
+    </row>
+    <row r="12" ht="102" customHeight="1">
+      <c r="A12" s="7" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="B12" s="6" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <b val="1"/>
-              <color rgb="0014322B"/>
-              <sz val="13"/>
-            </rPr>
-            <t>Regional background: Vietnam nine-month realized FDI rises 12.1%; distinguish registrations from execution</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <color rgb="007A8780"/>
-              <sz val="11"/>
-            </rPr>
-            <t xml:space="preserve">   Oct 17
+      <c r="B12" s="8" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="0014322B"/>
+              <sz val="13"/>
+            </rPr>
+            <t xml:space="preserve">Regional background: Vietnam nine-month realized FDI rises 12.1%; distinguish registrations from execution
 </t>
           </r>
           <r>
@@ -852,11 +839,14 @@
             <t>Vietnam’s government news portal reported October 3 that estimated realized FDI reached $21.07 billion in the first nine months, up 12.1% yearly, while total registered foreign investment reached $50.36 billion, up 76.4%. This is regional background through September 30, not a new October 17 release.</t>
           </r>
         </is>
+      </c>
+      <c r="C12" s="9" t="n">
+        <v>46298</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="A1:C1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" fitToHeight="0" fitToWidth="1"/>
@@ -870,11 +860,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:B12"/>
+  <dimension ref="A1:C12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="92" customWidth="1" min="2" max="2"/>
+    <col width="86" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1" ht="40" customHeight="1">
@@ -884,34 +875,39 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="6" customHeight="1">
-      <c r="A2" s="2" t="n"/>
-      <c r="B2" s="2" t="n"/>
-    </row>
-    <row r="3" ht="254" customHeight="1">
-      <c r="A3" s="3" t="inlineStr">
+    <row r="2" ht="22" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>Story</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Event date</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="274" customHeight="1">
+      <c r="A3" s="4" t="inlineStr">
         <is>
           <t>01</t>
         </is>
       </c>
-      <c r="B3" s="4" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <b val="1"/>
-              <color rgb="0014322B"/>
-              <sz val="13"/>
-            </rPr>
-            <t>Weekly follow-up: TSMC CoWoS production and Micron’s Taichung HBM assembly/test opening</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <color rgb="007A8780"/>
-              <sz val="11"/>
-            </rPr>
-            <t xml:space="preserve">   Oct 17
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="0014322B"/>
+              <sz val="13"/>
+            </rPr>
+            <t xml:space="preserve">Weekly follow-up: TSMC CoWoS production and Micron’s Taichung HBM assembly/test opening
 </t>
           </r>
           <r>
@@ -924,31 +920,26 @@
           </r>
         </is>
       </c>
-    </row>
-    <row r="4" ht="254" customHeight="1">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="C3" s="6" t="n">
+        <v>46310</v>
+      </c>
+    </row>
+    <row r="4" ht="274" customHeight="1">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>02</t>
         </is>
       </c>
-      <c r="B4" s="4" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <b val="1"/>
-              <color rgb="0014322B"/>
-              <sz val="13"/>
-            </rPr>
-            <t>Taiwan vendors exhibit racks, 800 VDC power and liquid cooling at OCP in San Jose</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <color rgb="007A8780"/>
-              <sz val="11"/>
-            </rPr>
-            <t xml:space="preserve">   Oct 17
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="0014322B"/>
+              <sz val="13"/>
+            </rPr>
+            <t xml:space="preserve">Taiwan vendors exhibit racks, 800 VDC power and liquid cooling at OCP in San Jose
 </t>
           </r>
           <r>
@@ -961,31 +952,26 @@
           </r>
         </is>
       </c>
-    </row>
-    <row r="5" ht="190" customHeight="1">
-      <c r="A5" s="3" t="inlineStr">
+      <c r="C4" s="6" t="n">
+        <v>46310</v>
+      </c>
+    </row>
+    <row r="5" ht="210" customHeight="1">
+      <c r="A5" s="4" t="inlineStr">
         <is>
           <t>03</t>
         </is>
       </c>
-      <c r="B5" s="4" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <b val="1"/>
-              <color rgb="0014322B"/>
-              <sz val="13"/>
-            </rPr>
-            <t>Ho Chi Minh City seeks clarity on AI data-center power tariffs</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <color rgb="007A8780"/>
-              <sz val="11"/>
-            </rPr>
-            <t xml:space="preserve">   Oct 17
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="0014322B"/>
+              <sz val="13"/>
+            </rPr>
+            <t xml:space="preserve">Ho Chi Minh City seeks clarity on AI data-center power tariffs
 </t>
           </r>
           <r>
@@ -998,31 +984,26 @@
           </r>
         </is>
       </c>
-    </row>
-    <row r="6" ht="178" customHeight="1">
-      <c r="A6" s="5" t="inlineStr">
+      <c r="C5" s="6" t="n">
+        <v>46310</v>
+      </c>
+    </row>
+    <row r="6" ht="198" customHeight="1">
+      <c r="A6" s="7" t="inlineStr">
         <is>
           <t>04</t>
         </is>
       </c>
-      <c r="B6" s="6" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <b val="1"/>
-              <color rgb="0014322B"/>
-              <sz val="13"/>
-            </rPr>
-            <t>Background follow-up: NVIDIA announces semiconductor inspection, testing and factory AI collaborations</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <color rgb="007A8780"/>
-              <sz val="11"/>
-            </rPr>
-            <t xml:space="preserve">   Oct 17
+      <c r="B6" s="8" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="0014322B"/>
+              <sz val="13"/>
+            </rPr>
+            <t xml:space="preserve">Background follow-up: NVIDIA announces semiconductor inspection, testing and factory AI collaborations
 </t>
           </r>
           <r>
@@ -1035,31 +1016,26 @@
           </r>
         </is>
       </c>
-    </row>
-    <row r="7" ht="222" customHeight="1">
-      <c r="A7" s="5" t="inlineStr">
+      <c r="C6" s="9" t="n">
+        <v>46309</v>
+      </c>
+    </row>
+    <row r="7" ht="242" customHeight="1">
+      <c r="A7" s="7" t="inlineStr">
         <is>
           <t>05</t>
         </is>
       </c>
-      <c r="B7" s="6" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <b val="1"/>
-              <color rgb="0014322B"/>
-              <sz val="13"/>
-            </rPr>
-            <t>Malaysia semiconductor recruitment spans process, equipment and facilities roles</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <color rgb="007A8780"/>
-              <sz val="11"/>
-            </rPr>
-            <t xml:space="preserve">   Oct 17
+      <c r="B7" s="8" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="0014322B"/>
+              <sz val="13"/>
+            </rPr>
+            <t xml:space="preserve">Malaysia semiconductor recruitment spans process, equipment and facilities roles
 </t>
           </r>
           <r>
@@ -1072,31 +1048,26 @@
           </r>
         </is>
       </c>
-    </row>
-    <row r="8" ht="174" customHeight="1">
-      <c r="A8" s="5" t="inlineStr">
+      <c r="C7" s="9" t="n">
+        <v>46311</v>
+      </c>
+    </row>
+    <row r="8" ht="178" customHeight="1">
+      <c r="A8" s="7" t="inlineStr">
         <is>
           <t>06</t>
         </is>
       </c>
-      <c r="B8" s="6" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <b val="1"/>
-              <color rgb="0014322B"/>
-              <sz val="13"/>
-            </rPr>
-            <t>AUO targets glass and optical components; pure-panel revenue share goal is 30% by 2030</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <color rgb="007A8780"/>
-              <sz val="11"/>
-            </rPr>
-            <t xml:space="preserve">   Oct 17
+      <c r="B8" s="8" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="0014322B"/>
+              <sz val="13"/>
+            </rPr>
+            <t xml:space="preserve">AUO targets glass and optical components; pure-panel revenue share goal is 30% by 2030
 </t>
           </r>
           <r>
@@ -1109,31 +1080,26 @@
           </r>
         </is>
       </c>
-    </row>
-    <row r="9" ht="146" customHeight="1">
-      <c r="A9" s="5" t="inlineStr">
+      <c r="C8" s="9" t="n">
+        <v>46312</v>
+      </c>
+    </row>
+    <row r="9" ht="166" customHeight="1">
+      <c r="A9" s="7" t="inlineStr">
         <is>
           <t>07</t>
         </is>
       </c>
-      <c r="B9" s="6" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <b val="1"/>
-              <color rgb="0014322B"/>
-              <sz val="13"/>
-            </rPr>
-            <t>RTX Spark PCs launch October 16, connecting Taiwan design, packaging and brands to local AI</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <color rgb="007A8780"/>
-              <sz val="11"/>
-            </rPr>
-            <t xml:space="preserve">   Oct 17
+      <c r="B9" s="8" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="0014322B"/>
+              <sz val="13"/>
+            </rPr>
+            <t xml:space="preserve">RTX Spark PCs launch October 16, connecting Taiwan design, packaging and brands to local AI
 </t>
           </r>
           <r>
@@ -1146,31 +1112,26 @@
           </r>
         </is>
       </c>
+      <c r="C9" s="9" t="n">
+        <v>46311</v>
+      </c>
     </row>
     <row r="10" ht="178" customHeight="1">
-      <c r="A10" s="5" t="inlineStr">
+      <c r="A10" s="7" t="inlineStr">
         <is>
           <t>08</t>
         </is>
       </c>
-      <c r="B10" s="6" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <b val="1"/>
-              <color rgb="0014322B"/>
-              <sz val="13"/>
-            </rPr>
-            <t>Taiwan says planned U.S. parks would be privately funded at an estimated $2–4 billion each</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <color rgb="007A8780"/>
-              <sz val="11"/>
-            </rPr>
-            <t xml:space="preserve">   Oct 17
+      <c r="B10" s="8" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="0014322B"/>
+              <sz val="13"/>
+            </rPr>
+            <t xml:space="preserve">Taiwan says planned U.S. parks would be privately funded at an estimated $2–4 billion each
 </t>
           </r>
           <r>
@@ -1183,31 +1144,26 @@
           </r>
         </is>
       </c>
-    </row>
-    <row r="11" ht="178" customHeight="1">
-      <c r="A11" s="5" t="inlineStr">
+      <c r="C10" s="9" t="n">
+        <v>46311</v>
+      </c>
+    </row>
+    <row r="11" ht="182" customHeight="1">
+      <c r="A11" s="7" t="inlineStr">
         <is>
           <t>09</t>
         </is>
       </c>
-      <c r="B11" s="6" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <b val="1"/>
-              <color rgb="0014322B"/>
-              <sz val="13"/>
-            </rPr>
-            <t>CIER raises Taiwan’s full-year growth forecast to 12.16%; distinguish results from projections</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <color rgb="007A8780"/>
-              <sz val="11"/>
-            </rPr>
-            <t xml:space="preserve">   Oct 17
+      <c r="B11" s="8" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="0014322B"/>
+              <sz val="13"/>
+            </rPr>
+            <t xml:space="preserve">CIER raises Taiwan’s full-year growth forecast to 12.16%; distinguish results from projections
 </t>
           </r>
           <r>
@@ -1220,31 +1176,26 @@
           </r>
         </is>
       </c>
-    </row>
-    <row r="12" ht="226" customHeight="1">
-      <c r="A12" s="5" t="inlineStr">
+      <c r="C11" s="9" t="n">
+        <v>46311</v>
+      </c>
+    </row>
+    <row r="12" ht="246" customHeight="1">
+      <c r="A12" s="7" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="B12" s="6" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <b val="1"/>
-              <color rgb="0014322B"/>
-              <sz val="13"/>
-            </rPr>
-            <t>Regional background: Vietnam nine-month realized FDI rises 12.1%; distinguish registrations from execution</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <color rgb="007A8780"/>
-              <sz val="11"/>
-            </rPr>
-            <t xml:space="preserve">   Oct 17
+      <c r="B12" s="8" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="0014322B"/>
+              <sz val="13"/>
+            </rPr>
+            <t xml:space="preserve">Regional background: Vietnam nine-month realized FDI rises 12.1%; distinguish registrations from execution
 </t>
           </r>
           <r>
@@ -1256,11 +1207,14 @@
             <t>Vietnam’s government news portal reported October 3 that estimated realized FDI reached $21.07 billion in the first nine months, up 12.1% yearly, while total registered foreign investment reached $50.36 billion, up 76.4%. This is regional background through September 30, not a new October 17 release. Location: Nationwide Vietnam statistics; not a single event or factory. Registrations include new projects, additions and equity transactions, while realized FDI uses a different scope. They cannot be added, and the ratio is not a project completion rate because cohorts differ. Comparable prior-year amounts are not provided. Manufacturing and investor-origin details lack original-table verification; realized FDI is estimated. VnEconomy reported October 4 that manufacturing and processing received $21.82 billion, or 50.3% of new and additional registrations. Singapore supplied $9.26 billion, or 31.7% of newly registered capital. Neither percentage uses the $50.36 billion total-registration denominator. These breakdowns have not been checked against original official tables and are source-limited. Nine-month realized FDI growth: 12.1% YoY. Verification confidence: Medium: official totals; added breakdowns await original-table verification.</t>
           </r>
         </is>
+      </c>
+      <c r="C12" s="9" t="n">
+        <v>46298</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="A1:C1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" fitToHeight="0" fitToWidth="1"/>

</xml_diff>

<commit_message>
feat(excel): add CEO lens column to the full sheet
Readers asked how a precision power and measurement company CEO might
read each story. The full sheet now shows story.ceoView in a separate,
clearly labelled AI-analysis column; the website stays facts-only.
The prompt also adds a 72-hour freshness rule for daily stories.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/exports/day-2026-10-17-en.xlsx
+++ b/docs/exports/day-2026-10-17-en.xlsx
@@ -24,7 +24,7 @@
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
     <numFmt numFmtId="165" formatCode="mmm d"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -56,8 +56,13 @@
       <color rgb="003B4A44"/>
       <sz val="11"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="003B4A44"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -72,6 +77,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF8E8"/>
       </patternFill>
     </fill>
   </fills>
@@ -97,7 +107,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -125,6 +135,9 @@
     </xf>
     <xf numFmtId="165" fontId="4" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -860,18 +873,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:C12"/>
+  <dimension ref="A1:D12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
     <col width="86" customWidth="1" min="2" max="2"/>
     <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="52" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1" ht="40" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Daily Brief highlights · 2026-10-17</t>
+          <t>Daily Brief full edition · 2026-10-17</t>
         </is>
       </c>
     </row>
@@ -891,6 +905,11 @@
           <t>Event date</t>
         </is>
       </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>CEO lens (AI analysis, not fact)</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="274" customHeight="1">
       <c r="A3" s="4" t="inlineStr">
@@ -923,6 +942,11 @@
       <c r="C3" s="6" t="n">
         <v>46310</v>
       </c>
+      <c r="D3" s="10" t="inlineStr">
+        <is>
+          <t>TSMC's CoWoS production and Micron's HBM assembly-and-test opening point to continued demand for plasma and RF power in etch, deposition and advanced packaging. A CEO would ask whether Taiwanese customers' tool delivery schedules track this capacity, which processes need tighter power control, and whether local service and spares can support new-fab ramps. Added output is undisclosed, so customer orders and tool-delivery timing are the evidence to watch, not a revenue estimate.</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="274" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
@@ -955,6 +979,11 @@
       <c r="C4" s="6" t="n">
         <v>46310</v>
       </c>
+      <c r="D4" s="10" t="inlineStr">
+        <is>
+          <t>800 VDC rack power and liquid cooling led Taiwanese exhibits, signalling a shift toward high-voltage DC in data-center power. For a power-conversion maker the questions are efficiency, power density and qualification timing, and whether Delta or Lite-On are competitors or partners. A CEO would check whether the roadmap covers 800 V architectures and whether joint validation with ODMs and cloud customers is needed; exhibits are not production orders.</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="210" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
@@ -987,6 +1016,11 @@
       <c r="C5" s="6" t="n">
         <v>46310</v>
       </c>
+      <c r="D5" s="10" t="inlineStr">
+        <is>
+          <t>Unsettled data-center tariffs in Ho Chi Minh City affect the cost and timing of local AI data centers. Higher tariffs make conversion efficiency and energy management more valuable, which favours high-efficiency power products, but project scale and timing remain uncertain. A CEO would keep Vietnam on a watch list until tariffs and the 50 MW first-phase timeline are clear.</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="198" customHeight="1">
       <c r="A6" s="7" t="inlineStr">
@@ -1019,6 +1053,11 @@
       <c r="C6" s="9" t="n">
         <v>46309</v>
       </c>
+      <c r="D6" s="10" t="inlineStr">
+        <is>
+          <t>NVIDIA's work with KLA, Advantest and factory-automation firms shows factory AI depends on rich tool data and real-time control. For precision measurement and control instruments, data interfaces, programmability and real-time feedback may become product requirements. A CEO would assess whether products can supply such data and whether to join these ecosystems, though deployments and benefits are not yet fully disclosed.</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="242" customHeight="1">
       <c r="A7" s="7" t="inlineStr">
@@ -1051,6 +1090,11 @@
       <c r="C7" s="9" t="n">
         <v>46311</v>
       </c>
+      <c r="D7" s="10" t="inlineStr">
+        <is>
+          <t>Malaysia's push to hire design, process, equipment and facilities staff reflects growing back-end and design clusters. For a tool supplier that means more local customers and installed tools, and tighter competition for engineering and service talent. A CEO would review Malaysian service coverage and staffing, and partnerships with local universities and parks for training.</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="178" customHeight="1">
       <c r="A8" s="7" t="inlineStr">
@@ -1083,6 +1127,11 @@
       <c r="C8" s="9" t="n">
         <v>46312</v>
       </c>
+      <c r="D8" s="10" t="inlineStr">
+        <is>
+          <t>A panel maker moving into glass substrates and TGV packaging parts could widen the supply base for advanced-packaging materials. Glass processing, laser drilling and coating also rely on stable plasma and precision power control, so a CEO might see a new process-tool customer group. Volume production is two to three years out and customer qualification is unconfirmed, so early technical contact and tracking qualification fit better than near-term plans.</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="166" customHeight="1">
       <c r="A9" s="7" t="inlineStr">
@@ -1115,6 +1164,11 @@
       <c r="C9" s="9" t="n">
         <v>46311</v>
       </c>
+      <c r="D9" s="10" t="inlineStr">
+        <is>
+          <t>AI PC launches mainly affect PC demand and relate only indirectly to precision power equipment, through added CoWoS demand upstream. A CEO would likely read it as AI demand spreading from data centers to devices and watch shipments rather than change strategy now.</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="178" customHeight="1">
       <c r="A10" s="7" t="inlineStr">
@@ -1147,6 +1201,11 @@
       <c r="C10" s="9" t="n">
         <v>46311</v>
       </c>
+      <c r="D10" s="10" t="inlineStr">
+        <is>
+          <t>Taiwanese industrial parks in Texas could add local electronics manufacturing and tool demand, letting a U.S.-based power and measurement company serve Taiwanese customers' U.S. sites up close. These are planning estimates with land, funding and tenants unconfirmed, so a CEO would first confirm existing Taiwanese customers' U.S. timelines before planning local sales and service.</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="182" customHeight="1">
       <c r="A11" s="7" t="inlineStr">
@@ -1179,6 +1238,11 @@
       <c r="C11" s="9" t="n">
         <v>46311</v>
       </c>
+      <c r="D11" s="10" t="inlineStr">
+        <is>
+          <t>Taiwan's growth forecast rising to 12.16%, driven by AI demand and corporate investment, suggests a still-strong capex environment among Taiwanese customers. A CEO would treat it as macro background alongside individual customer expansion plans, currency and geopolitical risk; forecasts can be revised and should not drive order expectations on their own.</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="246" customHeight="1">
       <c r="A12" s="7" t="inlineStr">
@@ -1211,12 +1275,17 @@
       <c r="C12" s="9" t="n">
         <v>46298</v>
       </c>
+      <c r="D12" s="10" t="inlineStr">
+        <is>
+          <t>Vietnam's registered FDI rose 76.4% with manufacturing about half, showing continued supply-chain diversification into Southeast Asia, but realized FDI grew only 12.1%, so execution lags commitments. A CEO would track which projects are semiconductor, electronics or data-center related and judge opportunity by actual construction and tool purchases, not registered amounts.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A1:D1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup orientation="portrait" fitToHeight="0" fitToWidth="1"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix(news): update 2026-10-17 verified coverage
Vietnam's nine-month FDI figures were released on October 3, two weeks
before this edition, so they read as stale news. The story moves into
industry context with its release date, the weekly theme now centres on
Ho Chi Minh City data-center tariffs, and the workbooks are rebuilt.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/exports/day-2026-10-17-en.xlsx
+++ b/docs/exports/day-2026-10-17-en.xlsx
@@ -505,7 +505,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:C12"/>
+  <dimension ref="A1:C11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -823,38 +823,6 @@
       </c>
       <c r="C11" s="9" t="n">
         <v>46311</v>
-      </c>
-    </row>
-    <row r="12" ht="102" customHeight="1">
-      <c r="A12" s="7" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="B12" s="8" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <b val="1"/>
-              <color rgb="0014322B"/>
-              <sz val="13"/>
-            </rPr>
-            <t xml:space="preserve">Regional background: Vietnam nine-month realized FDI rises 12.1%; distinguish registrations from execution
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <color rgb="003B4A44"/>
-              <sz val="11"/>
-            </rPr>
-            <t>Vietnam’s government news portal reported October 3 that estimated realized FDI reached $21.07 billion in the first nine months, up 12.1% yearly, while total registered foreign investment reached $50.36 billion, up 76.4%. This is regional background through September 30, not a new October 17 release.</t>
-          </r>
-        </is>
-      </c>
-      <c r="C12" s="9" t="n">
-        <v>46298</v>
       </c>
     </row>
   </sheetData>
@@ -873,7 +841,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D12"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1244,43 +1212,6 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="246" customHeight="1">
-      <c r="A12" s="7" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="B12" s="8" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <b val="1"/>
-              <color rgb="0014322B"/>
-              <sz val="13"/>
-            </rPr>
-            <t xml:space="preserve">Regional background: Vietnam nine-month realized FDI rises 12.1%; distinguish registrations from execution
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <color rgb="003B4A44"/>
-              <sz val="11"/>
-            </rPr>
-            <t>Vietnam’s government news portal reported October 3 that estimated realized FDI reached $21.07 billion in the first nine months, up 12.1% yearly, while total registered foreign investment reached $50.36 billion, up 76.4%. This is regional background through September 30, not a new October 17 release. Location: Nationwide Vietnam statistics; not a single event or factory. Registrations include new projects, additions and equity transactions, while realized FDI uses a different scope. They cannot be added, and the ratio is not a project completion rate because cohorts differ. Comparable prior-year amounts are not provided. Manufacturing and investor-origin details lack original-table verification; realized FDI is estimated. VnEconomy reported October 4 that manufacturing and processing received $21.82 billion, or 50.3% of new and additional registrations. Singapore supplied $9.26 billion, or 31.7% of newly registered capital. Neither percentage uses the $50.36 billion total-registration denominator. These breakdowns have not been checked against original official tables and are source-limited. Nine-month realized FDI growth: 12.1% YoY. Verification confidence: Medium: official totals; added breakdowns await original-table verification.</t>
-          </r>
-        </is>
-      </c>
-      <c r="C12" s="9" t="n">
-        <v>46298</v>
-      </c>
-      <c r="D12" s="10" t="inlineStr">
-        <is>
-          <t>Vietnam's registered FDI rose 76.4% with manufacturing about half, showing continued supply-chain diversification into Southeast Asia, but realized FDI grew only 12.1%, so execution lags commitments. A CEO would track which projects are semiconductor, electronics or data-center related and judge opportunity by actual construction and tool purchases, not registered amounts.</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:D1"/>

</xml_diff>

<commit_message>
fix(news): rewrite 2026-10-17 stories in a natural reading voice
Paragraphs read like audit notes: appended "label: value" lines,
repeated caveats and internal editing phrases. The edition now leads
with the news and gathers limitations at the end, without changing
facts. Paragraphs no longer append confidence or the headline figure;
location and confidence sit beside the headline, and the Excel column
is renamed AI 解讀.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/exports/day-2026-10-17-en.xlsx
+++ b/docs/exports/day-2026-10-17-en.xlsx
@@ -561,7 +561,7 @@
               <color rgb="003B4A44"/>
               <sz val="11"/>
             </rPr>
-            <t>TSMC said on October 15 that its five-reticle CoWoS platform was in production. Micron opened its Taichung AATT2 advanced assembly and test facility for HBM the same day. These are weekly follow-ups; no new capacity figures are established today.</t>
+            <t>TSMC said at its October 15 earnings call that its five-reticle CoWoS platform is in volume production. The same day, Micron opened its AATT2 advanced assembly and test plant in Taichung for HBM. Both are developments from earlier this week, and neither company disclosed added capacity.</t>
           </r>
         </is>
       </c>
@@ -593,7 +593,7 @@
               <color rgb="003B4A44"/>
               <sz val="11"/>
             </rPr>
-            <t>CNA’s October 17 roundup of the October 12–15 OCP summit in San Jose, California describes server or rack exhibits from Wiwynn, ASUS and Chenbro, alongside power systems from Delta, Lite-On and AcBel. Delta’s October 15 release details 800 VDC power, backup and liquid cooling products. Exhibits are distinct from production deployments.</t>
+            <t>According to CNA's October 17 roundup, Taiwanese suppliers featured prominently at the OCP Global Summit in San Jose on October 12–15: Wiwynn, ASUS and Chenbro showed new servers and racks, while Delta, Lite-On and AcBel focused on high-voltage DC power. Delta's October 15 release lists 800 VDC power racks, backup and liquid cooling, though these are exhibit specifications rather than production deployments.</t>
           </r>
         </is>
       </c>
@@ -601,7 +601,7 @@
         <v>46310</v>
       </c>
     </row>
-    <row r="5" ht="82" customHeight="1">
+    <row r="5" ht="98" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
           <t>03</t>
@@ -625,7 +625,7 @@
               <color rgb="003B4A44"/>
               <sz val="11"/>
             </rPr>
-            <t>TNGlobal reported October 16 that Ho Chi Minh City’s industrial-zone authority sought unified AI data-center power-tariff guidance at an October 15 meeting. The AIC–KBC project, with a planned $2.1 billion investment, was announced in March. The new development is tariff clarification, not a new investment announcement.</t>
+            <t>According to TNGlobal on October 16, Ho Chi Minh City's industrial-zone authority asked at an October 15 economic meeting for unified guidance on power tariffs for AI data centers. The related AIC–KBC project, with a planned US$2.1 billion investment, was announced in March; the new development is the tariff question, not new investment.</t>
           </r>
         </is>
       </c>
@@ -657,7 +657,7 @@
               <color rgb="003B4A44"/>
               <sz val="11"/>
             </rPr>
-            <t>NVIDIA’s October 14 release describes KLA inspection, Advantest testing and factory AI collaborations involving Foxconn and FANUC. This is background for Taiwan-linked supply chains and end-use factories; deployment sites, full production schedules and plant-wide ROI are not fully disclosed.</t>
+            <t>NVIDIA's October 14 release lists several collaborations: KLA inspection, Advantest testing, and factory AI work with Foxconn, FANUC and others. Released earlier this week, it does not fully disclose deployment sites, production timelines or plant-wide returns.</t>
           </r>
         </is>
       </c>
@@ -689,7 +689,7 @@
               <color rgb="003B4A44"/>
               <sz val="11"/>
             </rPr>
-            <t>CNA reported October 16 that a semiconductor recruitment event organized by Selangor-linked institutions at KLCC in Kuala Lumpur offered over 1,500 vacancies across design, software, firmware, process, equipment and facilities. An official reported 20 companies and 409 engineers in two design parks, complementing Penang manufacturing, assembly and testing.</t>
+            <t>CNA reported on October 16 that Selangor-linked institutions held a semiconductor recruitment event at the Kuala Lumpur Convention Centre (KLCC), offering more than 1,500 openings in design, software and firmware, process, equipment and facilities. An official said two IC design parks host 20 companies and 409 engineers, complementing Penang's manufacturing, assembly and testing.</t>
           </r>
         </is>
       </c>
@@ -721,7 +721,7 @@
               <color rgb="003B4A44"/>
               <sz val="11"/>
             </rPr>
-            <t>AUO chairman Paul Peng said on October 17 that the company would supply advanced-packaging components using glass and TGV expertise. Technology developed with Corning already has low-earth-orbit antenna applications. A two-to-three-year volume-production outlook for MicroLED optical communications and CPO remains a company forecast.</t>
+            <t>AUO chairman Paul Peng told CNA on October 17 that AUO will enter advanced-packaging components using glass and TGV (through-glass via) technology, and that technology developed with Corning is already used in low-earth-orbit satellite antennas. He expects MicroLED optical communications and CPO to reach volume production in about two to three years.</t>
           </r>
         </is>
       </c>
@@ -753,7 +753,7 @@
               <color rgb="003B4A44"/>
               <sz val="11"/>
             </rPr>
-            <t>NVIDIA announced RTX Spark Windows PCs on October 16, with ASUS, MSI and international PC brands using Grace CPUs and Blackwell GPUs. An executive told CNA that MediaTek contributed CPU design and that the platform uses CoWoS; demand and capacity assessments remain company statements.</t>
+            <t>NVIDIA launched RTX Spark Windows PCs on October 16, with ASUS, MSI and other brands offering models built on Grace CPUs and Blackwell GPUs. An NVIDIA executive told CNA that MediaTek contributed to the CPU design and that the platform uses CoWoS packaging.</t>
           </r>
         </is>
       </c>
@@ -785,7 +785,7 @@
               <color rgb="003B4A44"/>
               <sz val="11"/>
             </rPr>
-            <t>Taiwan’s economics ministry told CNA on October 16 that it would work with TEEMA on privately funded overseas industrial parks. Minister Kung Ming-hsin described starting in Texas; the estimated $2–4 billion per park is a plan, with land details unconfirmed.</t>
+            <t>Taiwan's Ministry of Economic Affairs told CNA on October 16 that it will work with TEEMA on overseas industrial parks funded by companies with government support. Minister Kung Ming-hsin said in an interview that the plan starts in Texas and will include more than one park, each estimated at US$2–4 billion.</t>
           </r>
         </is>
       </c>
@@ -793,7 +793,7 @@
         <v>46311</v>
       </c>
     </row>
-    <row r="11" ht="102" customHeight="1">
+    <row r="11" ht="86" customHeight="1">
       <c r="A11" s="7" t="inlineStr">
         <is>
           <t>09</t>
@@ -817,7 +817,7 @@
               <color rgb="003B4A44"/>
               <sz val="11"/>
             </rPr>
-            <t>CIER’s October 16 forecast raised 2026 growth from July’s 10.35% to 12.16%, an increase of 1.81 percentage points. Domestic demand is projected to contribute 6.63 points and net external demand 5.53; the full-year figure remains a forecast.</t>
+            <t>CIER's October 16 forecast raised Taiwan's 2026 GDP growth estimate from July's 10.35% to 12.16%, up 1.81 percentage points. Domestic demand is expected to contribute 6.63 points and net external demand 5.53 points.</t>
           </r>
         </is>
       </c>
@@ -875,11 +875,11 @@
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>CEO lens (AI analysis, not fact)</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="274" customHeight="1">
+          <t>AI interpretation</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="290" customHeight="1">
       <c r="A3" s="4" t="inlineStr">
         <is>
           <t>01</t>
@@ -903,7 +903,7 @@
               <color rgb="003B4A44"/>
               <sz val="11"/>
             </rPr>
-            <t>TSMC said on October 15 that its five-reticle CoWoS platform was in production. Micron opened its Taichung AATT2 advanced assembly and test facility for HBM the same day. These are weekly follow-ups; no new capacity figures are established today. Location: Micron opening: AATT2 advanced assembly and test facility, Taichung, Taiwan. AI designs move through wafer fabrication, packaging with HBM, testing and server assembly. Yield or delivery constraints at any layer can limit systems output; announced expansions cannot simply be added together. HBM serves accelerator packages, server DRAM system memory, and NAND and enterprise SSDs storage. TrendForce’s September 30 research describes stronger server and enterprise SSD demand alongside cautious consumer purchasing. This background forecast does not establish universal profit growth. Upstream checks include etch, deposition and equipment power; downstream checks include substrates, bonding, probes, burn-in and reliability. TrendForce’s October 13 mapping identifies Taiwanese testing or assembly roles including MPI, WinWay, Chroma and ASE. It does not establish new orders for these events. Added AATT2 HBM output, tool orders and individual supplier revenue are undisclosed. TSMC reported Q3 revenue of US$46.72 billion and a 66.4% gross margin. Taiwan-dollar revenue was about NT$1.494 trillion, up 50.9% annually, and net income NT$763.06 billion, up 68.7%. Growth rates in different currencies must remain distinct. These results were released October 15. From wafers to backend delivery: CoWoS / HBM. Verification confidence: High.</t>
+            <t>TSMC said at its October 15 earnings call that its five-reticle CoWoS platform is in volume production. The same day, Micron opened its AATT2 advanced assembly and test plant in Taichung for HBM. Both are developments from earlier this week, and neither company disclosed added capacity. AI chips start in wafer fabs, then are packaged with HBM and tested before server makers assemble them. A yield or lead-time problem at any step limits final shipments, so separate expansion announcements cannot simply be added up into usable systems. HBM goes into accelerator packages, server DRAM into system memory, and NAND and enterprise SSDs into storage. TrendForce's September 30 research saw stronger server and enterprise SSD demand but cautious consumer buying; that is a forecast, not evidence that every memory maker's profits are rising. Front-end processes rely on etch, deposition and tool power; back-end steps depend on substrates, bonding, probes, burn-in and reliability testing. TrendForce's October 13 map places Taiwan's MPI, WinWay, Chroma and ASE in testing and packaging roles, though it does not show new orders tied to these events. TSMC reported third-quarter results the same day: revenue of US$46.72 billion and a 66.4% gross margin; Taiwan-dollar revenue of about NT$1.494 trillion, up 50.9% year on year, and net income of NT$763.06 billion, up 68.7%. Growth rates in each currency are calculated separately and should not be mixed. AATT2's added HBM output, tool orders and any effect on individual suppliers' revenue have not been disclosed. Location: Micron AATT2 advanced assembly and test plant, Taichung, Taiwan.</t>
           </r>
         </is>
       </c>
@@ -916,7 +916,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="274" customHeight="1">
+    <row r="4" ht="226" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
         <is>
           <t>02</t>
@@ -940,7 +940,7 @@
               <color rgb="003B4A44"/>
               <sz val="11"/>
             </rPr>
-            <t>CNA’s October 17 roundup of the October 12–15 OCP summit in San Jose, California describes server or rack exhibits from Wiwynn, ASUS and Chenbro, alongside power systems from Delta, Lite-On and AcBel. Delta’s October 15 release details 800 VDC power, backup and liquid cooling products. Exhibits are distinct from production deployments. Location: San Jose McEnery Convention Center, San Jose, California, United States. OCP Global Summit 2026 ran October 12–15 local time in San Jose, California, at the San Jose McEnery Convention Center. Coverage follows Taiwanese exhibitors; the event location does not imply that their production or investment is located in the United States. Chips, HBM and packaging still need boards, networking, mechanics, power, backup, cooling and system testing. Availability and site power affect customer acceptance; compute specifications cover only part of delivery. Delta, Lite-On and AcBel exhibits make high-voltage DC design and integration comparable topics. Comparable costs, efficiency curves and production orders are unavailable, preventing market-share conclusions; product specifications and customer qualifications need separate comparisons. Delta lists a 660 kW power rack and 480 kW backup rating. These are product capabilities, not deployed customer consumption or sold capacity. The 800 V architecture is not an energy-saving percentage. Comparable prices, costs, customer orders and deployed volumes are undisclosed. Exhibited power architecture: 800 VDC. Verification confidence: High.</t>
+            <t>According to CNA's October 17 roundup, Taiwanese suppliers featured prominently at the OCP Global Summit in San Jose on October 12–15: Wiwynn, ASUS and Chenbro showed new servers and racks, while Delta, Lite-On and AcBel focused on high-voltage DC power. Delta's October 15 release lists 800 VDC power racks, backup and liquid cooling, though these are exhibit specifications rather than production deployments. After chips, HBM and packaging, a rack still needs boards, networking, mechanics, power, backup, cooling and system testing before it can ship. Customer acceptance therefore depends on availability and site power, not compute specifications alone. Delta lists a 660 kW power rack and a 480 kW backup rating; these are product ratings, not customers' actual consumption or sold capacity, and 800 V describes the architecture's voltage rather than an energy saving. With Delta, Lite-On and AcBel exhibiting side by side, high-voltage DC designs can now be compared, but comparable costs, efficiency curves and production orders are not public, so market-share shifts cannot yet be judged. Comparable prices, costs, customer orders and deployed volumes have not been disclosed. Location: San Jose McEnery Convention Center, San Jose, California, United States.</t>
           </r>
         </is>
       </c>
@@ -953,7 +953,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="210" customHeight="1">
+    <row r="5" ht="194" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
           <t>03</t>
@@ -977,7 +977,7 @@
               <color rgb="003B4A44"/>
               <sz val="11"/>
             </rPr>
-            <t>TNGlobal reported October 16 that Ho Chi Minh City’s industrial-zone authority sought unified AI data-center power-tariff guidance at an October 15 meeting. The AIC–KBC project, with a planned $2.1 billion investment, was announced in March. The new development is tariff clarification, not a new investment announcement. Location: Ho Chi Minh City, Vietnam; project at Tan Phu Trung Industrial Park. The issue is business versus manufacturing tariffs. Higher tariffs could affect costs, feasibility and timing. Final rates, load profiles and a financial model are unavailable, preventing a quantified cost difference. Original meeting records, final tariffs, load profiles and power contracts are unavailable. TNGlobal describes phase-one plans of up to 50 MW, while $2.1 billion refers to the previously announced overall project. Their scope and timing are not fully aligned. No per-MW construction cost is calculated from these figures, and planned capacity is not energized or leased capacity. Previously announced project amount: US$2.1B. Verification confidence: Medium.</t>
+            <t>According to TNGlobal on October 16, Ho Chi Minh City's industrial-zone authority asked at an October 15 economic meeting for unified guidance on power tariffs for AI data centers. The related AIC–KBC project, with a planned US$2.1 billion investment, was announced in March; the new development is the tariff question, not new investment. The question is whether data centers pay business or manufacturing tariffs. Higher tariffs would raise operating costs and could affect financial feasibility and construction timing, but final rates, load profiles and financial models are not public, so the cost difference cannot yet be estimated. TNGlobal cites up to 50 MW for phase one, while US$2.1 billion covers the whole project; their scope and timing differ, so dividing one by the other does not give a cost per MW, and planned capacity is not energized or leased capacity. Original meeting records, final tariffs, load profiles and power contracts are not yet available. Location: Tan Phu Trung Industrial Park, Ho Chi Minh City, Vietnam.</t>
           </r>
         </is>
       </c>
@@ -990,7 +990,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="198" customHeight="1">
+    <row r="6" ht="166" customHeight="1">
       <c r="A6" s="7" t="inlineStr">
         <is>
           <t>04</t>
@@ -1014,7 +1014,7 @@
               <color rgb="003B4A44"/>
               <sz val="11"/>
             </rPr>
-            <t>NVIDIA’s October 14 release describes KLA inspection, Advantest testing and factory AI collaborations involving Foxconn and FANUC. This is background for Taiwan-linked supply chains and end-use factories; deployment sites, full production schedules and plant-wide ROI are not fully disclosed. Location: Global collaboration announcement; individual factory deployment sites are not fully disclosed. Chips and servers provide compute, inspection and test tools generate data, and factories connect models to engineering, scheduling or operations. Partnership lists indicate possible interfaces; they do not establish complete integration or transferability across plants. Named deployment sites, contract pricing and quantified plant-wide benefits are incompletely disclosed. Track adoption; no verified plant-wide returns: 試點與驗收. Verification confidence: Medium.</t>
+            <t>NVIDIA's October 14 release lists several collaborations: KLA inspection, Advantest testing, and factory AI work with Foxconn, FANUC and others. Released earlier this week, it does not fully disclose deployment sites, production timelines or plant-wide returns. Chips and servers supply compute, inspection and test tools generate data, and factories feed models into engineering, scheduling and floor operations. The partner list shows how integration could work, but it does not prove every tool is connected or that the approach transfers to every plant. Named deployment sites, contract pricing and quantified plant-wide benefits have not been disclosed.</t>
           </r>
         </is>
       </c>
@@ -1027,7 +1027,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="242" customHeight="1">
+    <row r="7" ht="194" customHeight="1">
       <c r="A7" s="7" t="inlineStr">
         <is>
           <t>05</t>
@@ -1051,7 +1051,7 @@
               <color rgb="003B4A44"/>
               <sz val="11"/>
             </rPr>
-            <t>CNA reported October 16 that a semiconductor recruitment event organized by Selangor-linked institutions at KLCC in Kuala Lumpur offered over 1,500 vacancies across design, software, firmware, process, equipment and facilities. An official reported 20 companies and 409 engineers in two design parks, complementing Penang manufacturing, assembly and testing. Location: Kuala Lumpur Convention Centre (KLCC), Kuala Lumpur, Malaysia; organized by Selangor-linked institutions. The recruitment venue is KLCC in Kuala Lumpur, Malaysia, distinct from the organizing state of Selangor. Sidec and CNA list October 14–17, while ASEM’s recruitment page lists October 15–17. The venue agrees, but the subevent start date differs; that discrepancy is retained. Backend operations require process, test, maintenance and facilities staff; design clusters also need customers and manufacturing partners. Vacancies signal recruiting demand, not realized hires, output or payroll. Actual hiring and retention are undisclosed; park and program figures are official statements. CNA quoted an official describing a RM150 million program involving Selangor, Penang and the national investment institution. Current disbursement, foreign-capital share and funding timing are not listed; program size differs from new FDI flows. Advertised vacancies, not hires: &gt;1,500. Verification confidence: Medium.</t>
+            <t>CNA reported on October 16 that Selangor-linked institutions held a semiconductor recruitment event at the Kuala Lumpur Convention Centre (KLCC), offering more than 1,500 openings in design, software and firmware, process, equipment and facilities. An official said two IC design parks host 20 companies and 409 engineers, complementing Penang's manufacturing, assembly and testing. Back-end manufacturing depends on process, test, maintenance and facilities staff working together, and design clusters need customers and manufacturing partners. Openings show hiring demand, not actual new jobs, output or payroll. The official also described a RM150 million program involving Selangor, Penang and the national investment agency. Disbursement timing and the foreign share were not given; this is a program budget, not an FDI figure. Actual hires and retention have not been reported; organizer pages give October 14 or 15 as the start date, though they agree on the venue. Location: Kuala Lumpur Convention Centre (KLCC), Kuala Lumpur, Malaysia.</t>
           </r>
         </is>
       </c>
@@ -1088,7 +1088,7 @@
               <color rgb="003B4A44"/>
               <sz val="11"/>
             </rPr>
-            <t>AUO chairman Paul Peng said on October 17 that the company would supply advanced-packaging components using glass and TGV expertise. Technology developed with Corning already has low-earth-orbit antenna applications. A two-to-three-year volume-production outlook for MicroLED optical communications and CPO remains a company forecast. Glass processing can extend into new components, but packaging reliability, flatness and production yield require qualification. Progress in satellite applications does not establish semiconductor-packaging acceptance. The 30% figure is a targeted revenue mix in 2030, not a 30% revenue decline. Coverage relies on CNA’s named interview; transcripts, customer qualification and profitability evidence were unavailable. Source-limited. Pure-panel revenue share target: 2030 / 30%. Verification confidence: Medium. New-business profitability, customer qualifications and a full transcript are unavailable.</t>
+            <t>AUO chairman Paul Peng told CNA on October 17 that AUO will enter advanced-packaging components using glass and TGV (through-glass via) technology, and that technology developed with Corning is already used in low-earth-orbit satellite antennas. He expects MicroLED optical communications and CPO to reach volume production in about two to three years. A panel maker's glass-processing skills can extend into packaging parts, but packaging glass faces stricter reliability, flatness and yield requirements and still needs customer qualification; progress in satellite antennas does not amount to semiconductor-packaging approval. The 30% in the report is AUO's target for pure-panel revenue as a share of the total in 2030, not a 30% revenue decline. The information comes from a named interview; a transcript, customer qualification status and new-business profitability are not yet available.</t>
           </r>
         </is>
       </c>
@@ -1101,7 +1101,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="166" customHeight="1">
+    <row r="9" ht="150" customHeight="1">
       <c r="A9" s="7" t="inlineStr">
         <is>
           <t>07</t>
@@ -1125,7 +1125,7 @@
               <color rgb="003B4A44"/>
               <sz val="11"/>
             </rPr>
-            <t>NVIDIA announced RTX Spark Windows PCs on October 16, with ASUS, MSI and international PC brands using Grace CPUs and Blackwell GPUs. An executive told CNA that MediaTek contributed CPU design and that the platform uses CoWoS; demand and capacity assessments remain company statements. NVIDIA lists Grace CPUs, Blackwell GPUs and brands including ASUS and MSI. An executive told CNA that MediaTek contributed CPU design and the platform uses CoWoS; this edition does not establish HBM content. Shipments, utilization and full lifecycle costs are unavailable in this edition. Company-stated maximum unified memory: 128 GB. Verification confidence: High.</t>
+            <t>NVIDIA launched RTX Spark Windows PCs on October 16, with ASUS, MSI and other brands offering models built on Grace CPUs and Blackwell GPUs. An NVIDIA executive told CNA that MediaTek contributed to the CPU design and that the platform uses CoWoS packaging. The platform links Taiwan's chip design, advanced packaging and PC brands: MediaTek contributed CPU design, the platform uses CoWoS packaging, and ASUS and MSI build the end products. NVIDIA lists up to 128 GB of unified memory; demand and capacity claims come from NVIDIA, and HBM content is unconfirmed. Shipments, utilization and full lifecycle costs have not been disclosed.</t>
           </r>
         </is>
       </c>
@@ -1138,7 +1138,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="178" customHeight="1">
+    <row r="10" ht="146" customHeight="1">
       <c r="A10" s="7" t="inlineStr">
         <is>
           <t>08</t>
@@ -1162,7 +1162,7 @@
               <color rgb="003B4A44"/>
               <sz val="11"/>
             </rPr>
-            <t>Taiwan’s economics ministry told CNA on October 16 that it would work with TEEMA on privately funded overseas industrial parks. Minister Kung Ming-hsin described starting in Texas; the estimated $2–4 billion per park is a plan, with land details unconfirmed. Location: Investment plan: Texas, United States; specific park land remains unconfirmed. The ministry described private funding with government assistance and TEEMA participation. Plans would start in Texas and involve more than one park, at an estimated $2–4 billion per park. The estimate comes from the minister and ministry statements reported by media. Full financing, budget and land documents were unavailable; it is neither appropriated government spending nor fully committed capital. Developer, land, complete financing and tenant lists are unconfirmed. Planning estimate per park: US$2–4B. Verification confidence: Medium.</t>
+            <t>Taiwan's Ministry of Economic Affairs told CNA on October 16 that it will work with TEEMA on overseas industrial parks funded by companies with government support. Minister Kung Ming-hsin said in an interview that the plan starts in Texas and will include more than one park, each estimated at US$2–4 billion. The US$2–4 billion figure comes from the minister and ministry statements to media and is a planning estimate. Without financing, budget or land documents, it is neither appropriated government spending nor capital that companies have committed. The developer, land, full financing and tenant list have not been confirmed. Location: Texas, United States (planned; specific site not yet confirmed).</t>
           </r>
         </is>
       </c>
@@ -1175,7 +1175,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="182" customHeight="1">
+    <row r="11" ht="166" customHeight="1">
       <c r="A11" s="7" t="inlineStr">
         <is>
           <t>09</t>
@@ -1199,7 +1199,7 @@
               <color rgb="003B4A44"/>
               <sz val="11"/>
             </rPr>
-            <t>CIER’s October 16 forecast raised 2026 growth from July’s 10.35% to 12.16%, an increase of 1.81 percentage points. Domestic demand is projected to contribute 6.63 points and net external demand 5.53; the full-year figure remains a forecast. The two figures are different vintages of the same-year forecast, separated by 1.81 percentage points. Fourth-quarter growth is projected at 8.20% against a high prior-year base; slower growth does not itself mean output contracts. CIER cited AI demand, corporate expansion and domestic investment as forecast drivers, alongside financing, geopolitical and AI-cybersecurity uncertainties. These are the institution’s assumptions for its full-year forecast. Full-year GDP remains a forecast, subject to subsequent actual data. CIER 2026 full-year GDP growth forecast: 12.16%. Verification confidence: High.</t>
+            <t>CIER's October 16 forecast raised Taiwan's 2026 GDP growth estimate from July's 10.35% to 12.16%, up 1.81 percentage points. Domestic demand is expected to contribute 6.63 points and net external demand 5.53 points. CIER sees AI demand, corporate expansion and domestic investment as the main drivers, while flagging financing, geopolitical and AI-security uncertainties. 10.35% and 12.16% are two forecasts for the same year made at different times. Fourth-quarter growth is projected at 8.20% against a high base a year earlier; slower growth on its own does not mean output is shrinking. The full-year figure is still a forecast and may be revised once official data are released.</t>
           </r>
         </is>
       </c>

</xml_diff>

<commit_message>
fix(excel): phrase AI interpretation without referring to a CEO
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/exports/day-2026-10-17-en.xlsx
+++ b/docs/exports/day-2026-10-17-en.xlsx
@@ -912,7 +912,7 @@
       </c>
       <c r="D3" s="10" t="inlineStr">
         <is>
-          <t>TSMC's CoWoS production and Micron's HBM assembly-and-test opening point to continued demand for plasma and RF power in etch, deposition and advanced packaging. A CEO would ask whether Taiwanese customers' tool delivery schedules track this capacity, which processes need tighter power control, and whether local service and spares can support new-fab ramps. Added output is undisclosed, so customer orders and tool-delivery timing are the evidence to watch, not a revenue estimate.</t>
+          <t>TSMC's CoWoS production and Micron's HBM plant opening point to continued demand for plasma and RF power in etch, deposition and advanced packaging. Worth asking: do Taiwanese customers' tool delivery schedules track this capacity, which processes need tighter power control, and is local service and spares coverage ready for new-fab ramps? Added output is undisclosed, so customer orders and delivery timing are better evidence than a revenue estimate.</t>
         </is>
       </c>
     </row>
@@ -949,7 +949,7 @@
       </c>
       <c r="D4" s="10" t="inlineStr">
         <is>
-          <t>800 VDC rack power and liquid cooling led Taiwanese exhibits, signalling a shift toward high-voltage DC in data-center power. For a power-conversion maker the questions are efficiency, power density and qualification timing, and whether Delta or Lite-On are competitors or partners. A CEO would check whether the roadmap covers 800 V architectures and whether joint validation with ODMs and cloud customers is needed; exhibits are not production orders.</t>
+          <t>800 VDC rack power and liquid cooling led Taiwanese exhibits, signalling a shift toward high-voltage DC in data-center power. For power-conversion suppliers the questions are efficiency, power density and qualification timing, and whether Delta or Lite-On are competitors or partners. A useful check is whether product roadmaps cover 800 V architectures and need joint validation with ODMs and cloud customers; exhibits are not production orders.</t>
         </is>
       </c>
     </row>
@@ -986,7 +986,7 @@
       </c>
       <c r="D5" s="10" t="inlineStr">
         <is>
-          <t>Unsettled data-center tariffs in Ho Chi Minh City affect the cost and timing of local AI data centers. Higher tariffs make conversion efficiency and energy management more valuable, which favours high-efficiency power products, but project scale and timing remain uncertain. A CEO would keep Vietnam on a watch list until tariffs and the 50 MW first-phase timeline are clear.</t>
+          <t>Unsettled data-center tariffs in Ho Chi Minh City affect the cost and timing of local AI data centers. Higher tariffs make conversion efficiency and energy management more valuable, which favours high-efficiency power products, but project scale and timing remain uncertain. Vietnam fits a watch list until tariffs and the 50 MW first-phase timeline are clear.</t>
         </is>
       </c>
     </row>
@@ -1023,7 +1023,7 @@
       </c>
       <c r="D6" s="10" t="inlineStr">
         <is>
-          <t>NVIDIA's work with KLA, Advantest and factory-automation firms shows factory AI depends on rich tool data and real-time control. For precision measurement and control instruments, data interfaces, programmability and real-time feedback may become product requirements. A CEO would assess whether products can supply such data and whether to join these ecosystems, though deployments and benefits are not yet fully disclosed.</t>
+          <t>NVIDIA's work with KLA, Advantest and factory-automation firms shows factory AI depends on rich tool data and real-time control. For precision measurement and control instrument makers, data interfaces, programmability and real-time feedback may become product requirements. It is worth assessing whether products can supply such data and whether to join these ecosystems, though deployments and benefits are not yet fully disclosed.</t>
         </is>
       </c>
     </row>
@@ -1060,7 +1060,7 @@
       </c>
       <c r="D7" s="10" t="inlineStr">
         <is>
-          <t>Malaysia's push to hire design, process, equipment and facilities staff reflects growing back-end and design clusters. For a tool supplier that means more local customers and installed tools, and tighter competition for engineering and service talent. A CEO would review Malaysian service coverage and staffing, and partnerships with local universities and parks for training.</t>
+          <t>Malaysia's push to hire design, process, equipment and facilities staff reflects growing back-end and design clusters. For tool suppliers that means more local customers and installed tools, and tighter competition for engineering and service talent. Worth reviewing: Malaysian service coverage and staffing, and training partnerships with local universities and parks.</t>
         </is>
       </c>
     </row>
@@ -1097,7 +1097,7 @@
       </c>
       <c r="D8" s="10" t="inlineStr">
         <is>
-          <t>A panel maker moving into glass substrates and TGV packaging parts could widen the supply base for advanced-packaging materials. Glass processing, laser drilling and coating also rely on stable plasma and precision power control, so a CEO might see a new process-tool customer group. Volume production is two to three years out and customer qualification is unconfirmed, so early technical contact and tracking qualification fit better than near-term plans.</t>
+          <t>A panel maker moving into glass substrates and TGV packaging parts could widen the supply base for advanced-packaging materials. Glass processing, laser drilling and coating also rely on stable plasma and precision power control, so such makers could become a new process-tool customer group. Volume production is two to three years out and qualification is unconfirmed, so early technical contact and tracking qualification fit better than near-term plans.</t>
         </is>
       </c>
     </row>
@@ -1134,7 +1134,7 @@
       </c>
       <c r="D9" s="10" t="inlineStr">
         <is>
-          <t>AI PC launches mainly affect PC demand and relate only indirectly to precision power equipment, through added CoWoS demand upstream. A CEO would likely read it as AI demand spreading from data centers to devices and watch shipments rather than change strategy now.</t>
+          <t>AI PC launches mainly affect PC demand and relate only indirectly to precision power equipment, through added CoWoS demand upstream. It reads best as a sign of AI demand spreading from data centers to devices, worth tracking through shipments rather than acting on now.</t>
         </is>
       </c>
     </row>
@@ -1171,7 +1171,7 @@
       </c>
       <c r="D10" s="10" t="inlineStr">
         <is>
-          <t>Taiwanese industrial parks in Texas could add local electronics manufacturing and tool demand, letting a U.S.-based power and measurement company serve Taiwanese customers' U.S. sites up close. These are planning estimates with land, funding and tenants unconfirmed, so a CEO would first confirm existing Taiwanese customers' U.S. timelines before planning local sales and service.</t>
+          <t>Taiwanese industrial parks in Texas could add local electronics manufacturing and tool demand, letting U.S.-based power and measurement suppliers serve Taiwanese customers' U.S. sites up close. These are planning estimates with land, funding and tenants unconfirmed, so confirming existing Taiwanese customers' U.S. timelines comes before planning local sales and service.</t>
         </is>
       </c>
     </row>
@@ -1208,7 +1208,7 @@
       </c>
       <c r="D11" s="10" t="inlineStr">
         <is>
-          <t>Taiwan's growth forecast rising to 12.16%, driven by AI demand and corporate investment, suggests a still-strong capex environment among Taiwanese customers. A CEO would treat it as macro background alongside individual customer expansion plans, currency and geopolitical risk; forecasts can be revised and should not drive order expectations on their own.</t>
+          <t>Taiwan's growth forecast rising to 12.16%, driven by AI demand and corporate investment, suggests a still-strong capex environment among Taiwanese customers. It works best as macro background alongside individual customer expansion plans, currency and geopolitical risk; forecasts can be revised and should not drive order expectations on their own.</t>
         </is>
       </c>
     </row>

</xml_diff>